<commit_message>
Fix LinkedIn composer detection with Shadow DOM piercing and direct content script injection
</commit_message>
<xml_diff>
--- a/memory/linkedin_posts.xlsx
+++ b/memory/linkedin_posts.xlsx
@@ -69,7 +69,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -78,6 +78,9 @@
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -445,7 +448,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G5"/>
+  <dimension ref="A1:G18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -611,6 +614,383 @@
         </is>
       </c>
     </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>2026-03-08</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>project_showcase</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>I’ve seen it – the frustration of building on Base L2 with raw `web3.py`. Developers were spending h</t>
+        </is>
+      </c>
+      <c r="D6" s="4" t="inlineStr">
+        <is>
+          <t>generated</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr"/>
+      <c r="F6" s="2" t="inlineStr"/>
+      <c r="G6" s="2" t="inlineStr">
+        <is>
+          <t>local</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>2026-03-08</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>project_showcase</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>I’ve seen developers struggle with building robust applications on Base L2. Raw `web3.py` just doesn</t>
+        </is>
+      </c>
+      <c r="D7" s="4" t="inlineStr">
+        <is>
+          <t>generated</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr"/>
+      <c r="F7" s="2" t="inlineStr"/>
+      <c r="G7" s="2" t="inlineStr">
+        <is>
+          <t>local</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>2026-03-08</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>project_showcase</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>I’ve seen it – the frustration of building on Base L2 with raw `web3.py`. Developers were spending h</t>
+        </is>
+      </c>
+      <c r="D8" s="4" t="inlineStr">
+        <is>
+          <t>generated</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="inlineStr"/>
+      <c r="F8" s="2" t="inlineStr"/>
+      <c r="G8" s="2" t="inlineStr">
+        <is>
+          <t>local</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>2026-03-08</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>project_showcase</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>I’ve been wrestling with building reliable applications on Base L2, and I kept running into the same</t>
+        </is>
+      </c>
+      <c r="D9" s="4" t="inlineStr">
+        <is>
+          <t>generated</t>
+        </is>
+      </c>
+      <c r="E9" s="2" t="inlineStr"/>
+      <c r="F9" s="2" t="inlineStr"/>
+      <c r="G9" s="2" t="inlineStr">
+        <is>
+          <t>local</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>2026-03-08</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>project_showcase</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>I’ve been spending a lot of time building applications on Base L2, and I’ve seen firsthand the heada</t>
+        </is>
+      </c>
+      <c r="D10" s="4" t="inlineStr">
+        <is>
+          <t>generated</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="inlineStr"/>
+      <c r="F10" s="2" t="inlineStr"/>
+      <c r="G10" s="2" t="inlineStr">
+        <is>
+          <t>local</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>2026-03-08</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>project_showcase</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">I’ve been spending a lot of time building applications on Base, and I’ve seen a frustrating pattern </t>
+        </is>
+      </c>
+      <c r="D11" s="4" t="inlineStr">
+        <is>
+          <t>generated</t>
+        </is>
+      </c>
+      <c r="E11" s="2" t="inlineStr"/>
+      <c r="F11" s="2" t="inlineStr"/>
+      <c r="G11" s="2" t="inlineStr">
+        <is>
+          <t>local</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>2026-03-08</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>project_showcase</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>I’ve seen it happen time and again: developers building applications on Base L2 – Coinbase’s excitin</t>
+        </is>
+      </c>
+      <c r="D12" s="4" t="inlineStr">
+        <is>
+          <t>generated</t>
+        </is>
+      </c>
+      <c r="E12" s="2" t="inlineStr"/>
+      <c r="F12" s="2" t="inlineStr"/>
+      <c r="G12" s="2" t="inlineStr">
+        <is>
+          <t>local</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>2026-03-08</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>project_showcase</t>
+        </is>
+      </c>
+      <c r="C13" s="2" t="inlineStr">
+        <is>
+          <t>I’ve seen it – the frustration! Building production apps on Base L2 with raw `web3.py` can quickly t</t>
+        </is>
+      </c>
+      <c r="D13" s="4" t="inlineStr">
+        <is>
+          <t>generated</t>
+        </is>
+      </c>
+      <c r="E13" s="2" t="inlineStr"/>
+      <c r="F13" s="2" t="inlineStr"/>
+      <c r="G13" s="2" t="inlineStr">
+        <is>
+          <t>local</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>2026-03-08</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>project_showcase</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>I’ve been wrestling with a frustrating problem in the Base ecosystem – building reliable dApps on La</t>
+        </is>
+      </c>
+      <c r="D14" s="4" t="inlineStr">
+        <is>
+          <t>generated</t>
+        </is>
+      </c>
+      <c r="E14" s="2" t="inlineStr"/>
+      <c r="F14" s="2" t="inlineStr"/>
+      <c r="G14" s="2" t="inlineStr">
+        <is>
+          <t>local</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t>2026-03-09</t>
+        </is>
+      </c>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>project_showcase</t>
+        </is>
+      </c>
+      <c r="C15" s="2" t="inlineStr">
+        <is>
+          <t>I’ve been spending a lot of time building on Base L2, and let me tell you, the raw `web3.py` experie</t>
+        </is>
+      </c>
+      <c r="D15" s="4" t="inlineStr">
+        <is>
+          <t>generated</t>
+        </is>
+      </c>
+      <c r="E15" s="2" t="inlineStr"/>
+      <c r="F15" s="2" t="inlineStr"/>
+      <c r="G15" s="2" t="inlineStr">
+        <is>
+          <t>local</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>2026-03-09</t>
+        </is>
+      </c>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>project_showcase</t>
+        </is>
+      </c>
+      <c r="C16" s="2" t="inlineStr">
+        <is>
+          <t>I’ve seen developers wrestle with building efficient applications on Base L2, and it’s a frustrating</t>
+        </is>
+      </c>
+      <c r="D16" s="4" t="inlineStr">
+        <is>
+          <t>generated</t>
+        </is>
+      </c>
+      <c r="E16" s="2" t="inlineStr"/>
+      <c r="F16" s="2" t="inlineStr"/>
+      <c r="G16" s="2" t="inlineStr">
+        <is>
+          <t>local</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="inlineStr">
+        <is>
+          <t>2026-03-09</t>
+        </is>
+      </c>
+      <c r="B17" s="2" t="inlineStr">
+        <is>
+          <t>project_showcase</t>
+        </is>
+      </c>
+      <c r="C17" s="2" t="inlineStr">
+        <is>
+          <t>I’ve been wrestling with a frustrating problem in building applications on Base L2: the sheer amount</t>
+        </is>
+      </c>
+      <c r="D17" s="4" t="inlineStr">
+        <is>
+          <t>generated</t>
+        </is>
+      </c>
+      <c r="E17" s="2" t="inlineStr"/>
+      <c r="F17" s="2" t="inlineStr"/>
+      <c r="G17" s="2" t="inlineStr">
+        <is>
+          <t>local</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>2026-03-09</t>
+        </is>
+      </c>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t>project_showcase</t>
+        </is>
+      </c>
+      <c r="C18" s="2" t="inlineStr">
+        <is>
+          <t>I’ve been spending a lot of time building on Base L2, and let me tell you, wrestling with raw `web3.</t>
+        </is>
+      </c>
+      <c r="D18" s="4" t="inlineStr">
+        <is>
+          <t>generated</t>
+        </is>
+      </c>
+      <c r="E18" s="2" t="inlineStr"/>
+      <c r="F18" s="2" t="inlineStr"/>
+      <c r="G18" s="2" t="inlineStr">
+        <is>
+          <t>local</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>